<commit_message>
use wikidata id for queries
</commit_message>
<xml_diff>
--- a/assets/raw-data/ff-projects/ff-projects.xlsx
+++ b/assets/raw-data/ff-projects/ff-projects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HesseE\mex-extractors\assets\raw-data\ff-projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61669A6F-9AA6-49F0-BA0A-867A4446BDED}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E32170-58A3-4144-B863-3D19A7FA5838}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32760" yWindow="32760" windowWidth="15360" windowHeight="4080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="66">
   <si>
     <t>Zuwendungs-/ Auftraggeber</t>
   </si>
@@ -227,6 +227,9 @@
   </si>
   <si>
     <t>Skipped Laufzeiten</t>
+  </si>
+  <si>
+    <t>Robert Koch-Institut</t>
   </si>
 </sst>
 </file>
@@ -2104,7 +2107,7 @@
         <v>9</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="E2" s="29"/>
       <c r="F2" s="30" t="s">

</xml_diff>

<commit_message>
feature/mx-1747 use wikidata id for queries (#353)
### Added

- add settings for wikidata mapping

### Changes

- switch out wikidata query by names with query by id

---------

Signed-off-by: erichesse <hessee@rki.de>
Signed-off-by: erichesse <eric.hesse3@yahoo.de>
Co-authored-by: Nicolas Drebenstedt <897972+cutoffthetop@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/assets/raw-data/ff-projects/ff-projects.xlsx
+++ b/assets/raw-data/ff-projects/ff-projects.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HesseE\mex-extractors\assets\raw-data\ff-projects\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61669A6F-9AA6-49F0-BA0A-867A4446BDED}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E32170-58A3-4144-B863-3D19A7FA5838}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="32760" yWindow="32760" windowWidth="15360" windowHeight="4080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="66">
   <si>
     <t>Zuwendungs-/ Auftraggeber</t>
   </si>
@@ -227,6 +227,9 @@
   </si>
   <si>
     <t>Skipped Laufzeiten</t>
+  </si>
+  <si>
+    <t>Robert Koch-Institut</t>
   </si>
 </sst>
 </file>
@@ -2104,7 +2107,7 @@
         <v>9</v>
       </c>
       <c r="D2" s="28" t="s">
-        <v>12</v>
+        <v>65</v>
       </c>
       <c r="E2" s="29"/>
       <c r="F2" s="30" t="s">

</xml_diff>